<commit_message>
Rebuild the demo workbook for the current output format
Adds Attempt and Status to Execution Metrics and the Unfinished sheet,
drops ErrorCode, updates the Finalization text. Numbers are unchanged;
names stay anonymised.
</commit_message>
<xml_diff>
--- a/demo/refresh_analysis_demo.xlsx
+++ b/demo/refresh_analysis_demo.xlsx
@@ -12,13 +12,14 @@
     <sheet name="System Events" sheetId="3" r:id="rId3"/>
     <sheet name="Errors" sheetId="4" r:id="rId4"/>
     <sheet name="Execution Metrics" sheetId="5" r:id="rId5"/>
+    <sheet name="Unfinished" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="177">
   <si>
     <t>Database</t>
   </si>
@@ -482,7 +483,7 @@
     <t>From the refresh command start to the first Timeline operation</t>
   </si>
   <si>
-    <t>Wait before Commit/Rollback and the tail after it (remainder of the refresh duration)</t>
+    <t>Wait before Commit and the tail after it (remainder of the refresh duration)</t>
   </si>
   <si>
     <t>ID</t>
@@ -491,9 +492,6 @@
     <t>Error</t>
   </si>
   <si>
-    <t>ErrorCode</t>
-  </si>
-  <si>
     <t>Command Type</t>
   </si>
   <si>
@@ -515,18 +513,59 @@
     <t>VertiPaq CPU Sec</t>
   </si>
   <si>
+    <t>Attempt</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
     <t>Batch</t>
   </si>
   <si>
     <t>2026-09-08 14:09:51.262</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>EventSubclass</t>
+  </si>
+  <si>
+    <t>Open_Until_Trace_End_Sec</t>
+  </si>
+  <si>
+    <t>b005d05a-7d8e-0b28-7367-dd8d59990b4b</t>
+  </si>
+  <si>
+    <t>ffe6319d-fdea-6ba0-2ffb-95b8038425c0</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>Building and preparing relationship for the 'Sales' table started. (TableTMID='16')</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:07:38.000</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:07:47.000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -542,7 +581,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -550,12 +589,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -854,16 +911,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -892,31 +949,31 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
@@ -3164,19 +3221,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>145</v>
       </c>
     </row>
@@ -3249,29 +3306,26 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="E1" t="s">
-        <v>157</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="F1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
@@ -3282,44 +3336,50 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" t="s">
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="H1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="L1" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B2">
         <v>6</v>
@@ -3343,9 +3403,85 @@
         <v>150</v>
       </c>
       <c r="I2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J2" t="s">
+        <v>143</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E2">
+        <v>133.157</v>
+      </c>
+      <c r="F2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3">
+        <v>124.157</v>
+      </c>
+      <c r="F3" t="s">
         <v>143</v>
       </c>
     </row>

</xml_diff>